<commit_message>
This is 2nd commit
</commit_message>
<xml_diff>
--- a/target/test-classes/TestData.xlsx
+++ b/target/test-classes/TestData.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="23">
   <si>
     <t>Username</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>PASS</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
 </sst>
 </file>
@@ -121,7 +124,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -138,6 +141,16 @@
         <fgColor indexed="17"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -151,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -188,6 +201,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
@@ -537,8 +554,8 @@
       <c r="C2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" t="s" s="28">
-        <v>21</v>
+      <c r="D2" t="s" s="35">
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -551,7 +568,7 @@
       <c r="C3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s" s="32">
+      <c r="D3" t="s" s="36">
         <v>21</v>
       </c>
     </row>
@@ -565,7 +582,7 @@
       <c r="C4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D4" t="s" s="33">
+      <c r="D4" t="s" s="37">
         <v>21</v>
       </c>
     </row>
@@ -573,7 +590,7 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
-      <c r="D5" t="s" s="34">
+      <c r="D5" t="s" s="38">
         <v>21</v>
       </c>
     </row>

</xml_diff>